<commit_message>
End of section 6
</commit_message>
<xml_diff>
--- a/lernzeiten_tracker.xlsx
+++ b/lernzeiten_tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A.Alzoubi\source\repos\demo\DatingApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{322D3849-E4A0-4BE1-89A0-49565A31D1FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44086AA2-7206-4A02-86BE-BE471CFAF191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-9670" yWindow="5310" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lernzeiten" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>Datum</t>
   </si>
@@ -67,6 +67,15 @@
   </si>
   <si>
     <t>Nav bar styling, Account service,homepage(Registerform)</t>
+  </si>
+  <si>
+    <t>Parent tu child communiction und umgekehrt, Register commponent an API schließen, Routing funktionalität hinzugefüg, Toast meldung hinzugefügt</t>
+  </si>
+  <si>
+    <t>Summe:</t>
+  </si>
+  <si>
+    <t>Route guard, app initialization, route Animations hinzugefügt</t>
   </si>
 </sst>
 </file>
@@ -437,7 +446,7 @@
                   <c:v>3.9999999999999991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.9999999999999991</c:v>
+                  <c:v>6.9999999999999982</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3.9999999999999991</c:v>
@@ -1510,8 +1519,8 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="86" customWidth="1"/>
+    <col min="5" max="5" width="11.85546875" customWidth="1"/>
+    <col min="6" max="6" width="141.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1604,15 +1613,39 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>46093</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="C6" s="4">
+        <v>0.54166666666666663</v>
+      </c>
       <c r="D6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2.9999999999999987</v>
+      </c>
+      <c r="E6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
+        <v>46094</v>
+      </c>
+      <c r="B7" s="4">
+        <v>0.39583333333333331</v>
+      </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-9.5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2789,7 +2822,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2819,7 +2852,7 @@
       </c>
       <c r="B3">
         <f>SUMIF(Lernzeiten!E:E,A3,Lernzeiten!D:D)</f>
-        <v>3.9999999999999991</v>
+        <v>6.9999999999999982</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2829,6 +2862,15 @@
       <c r="B4">
         <f>SUMIF(Lernzeiten!E:E,A4,Lernzeiten!D:D)</f>
         <v>3.9999999999999991</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <f>SUM(B2:B5)</f>
+        <v>14.999999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
End of section 7
</commit_message>
<xml_diff>
--- a/lernzeiten_tracker.xlsx
+++ b/lernzeiten_tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A.Alzoubi\source\repos\demo\DatingApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44086AA2-7206-4A02-86BE-BE471CFAF191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502812F7-A70C-4665-8D03-53AFA2AEFFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-9670" yWindow="5310" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -75,7 +75,7 @@
     <t>Summe:</t>
   </si>
   <si>
-    <t>Route guard, app initialization, route Animations hinzugefügt</t>
+    <t>(Route guard, app initialization, route Animations hinzugefügt)</t>
   </si>
 </sst>
 </file>
@@ -446,10 +446,10 @@
                   <c:v>3.9999999999999991</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6.9999999999999982</c:v>
+                  <c:v>8.4999999999999982</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.9999999999999991</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1566,9 +1566,6 @@
         <f t="shared" ref="D3:D33" si="0">(C3-B3)*24</f>
         <v>3.9999999999999991</v>
       </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
@@ -1640,9 +1637,15 @@
       <c r="B7" s="4">
         <v>0.39583333333333331</v>
       </c>
+      <c r="C7" s="4">
+        <v>0.45833333333333331</v>
+      </c>
       <c r="D7">
         <f t="shared" si="0"/>
-        <v>-9.5</v>
+        <v>1.5</v>
+      </c>
+      <c r="E7" t="s">
+        <v>7</v>
       </c>
       <c r="F7" t="s">
         <v>13</v>
@@ -2852,7 +2855,7 @@
       </c>
       <c r="B3">
         <f>SUMIF(Lernzeiten!E:E,A3,Lernzeiten!D:D)</f>
-        <v>6.9999999999999982</v>
+        <v>8.4999999999999982</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -2861,7 +2864,7 @@
       </c>
       <c r="B4">
         <f>SUMIF(Lernzeiten!E:E,A4,Lernzeiten!D:D)</f>
-        <v>3.9999999999999991</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -2870,7 +2873,7 @@
       </c>
       <c r="B6">
         <f>SUM(B2:B5)</f>
-        <v>14.999999999999996</v>
+        <v>12.499999999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>